<commit_message>
Clean code, update wind rose source file
</commit_message>
<xml_diff>
--- a/data/WindResource.xlsx
+++ b/data/WindResource.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Software\IEA-Wind-2200-22-ROWP\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB7F100C-44DC-441E-81DF-DF1427C6CFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60B5E9E2-0893-4A85-80AB-7D0AAD41CD2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1860" windowWidth="29040" windowHeight="17640" xr2:uid="{B2AF22FD-04A2-44E7-8A6F-3F4AE8E78B84}"/>
+    <workbookView xWindow="13800" yWindow="0" windowWidth="14057" windowHeight="17880" xr2:uid="{B2AF22FD-04A2-44E7-8A6F-3F4AE8E78B84}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
   <si>
     <t>Sector</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>at 170m (Hub Height)</t>
+  </si>
+  <si>
+    <t>Taken from Table 50 in "Wind Resource Assessment Hollandse Kust (west) Wind Farm Zone Update February 2022"</t>
   </si>
 </sst>
 </file>
@@ -76,9 +79,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.00000"/>
+    <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -90,6 +93,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -115,10 +125,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -454,14 +465,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A2AE255-00A1-451F-AD6B-B207EFC19EAB}">
   <dimension ref="A1:M30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -480,8 +491,11 @@
       <c r="F2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="I2" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>0</v>
       </c>
@@ -501,7 +515,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>30</v>
       </c>
@@ -521,7 +535,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>60</v>
       </c>
@@ -541,7 +555,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>90</v>
       </c>
@@ -561,7 +575,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>120</v>
       </c>
@@ -590,7 +604,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>150</v>
       </c>
@@ -619,7 +633,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>180</v>
       </c>
@@ -639,7 +653,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>210</v>
       </c>
@@ -659,7 +673,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>240</v>
       </c>
@@ -679,7 +693,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>270</v>
       </c>
@@ -699,7 +713,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>300</v>
       </c>
@@ -719,7 +733,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>330</v>
       </c>
@@ -739,12 +753,12 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -761,7 +775,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>0</v>
       </c>
@@ -781,7 +795,7 @@
         <v>5.9800000000000006E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A20">
         <v>30</v>
       </c>
@@ -801,7 +815,7 @@
         <v>5.9400000000000001E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>60</v>
       </c>
@@ -821,7 +835,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A22">
         <v>90</v>
       </c>
@@ -841,7 +855,7 @@
         <v>6.6699999999999995E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A23">
         <v>120</v>
       </c>
@@ -861,7 +875,7 @@
         <v>4.9200000000000001E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>150</v>
       </c>
@@ -881,7 +895,7 @@
         <v>4.7800000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A25">
         <v>180</v>
       </c>
@@ -901,7 +915,7 @@
         <v>7.6399999999999996E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26">
         <v>210</v>
       </c>
@@ -921,7 +935,7 @@
         <v>0.1426</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>240</v>
       </c>
@@ -941,7 +955,7 @@
         <v>0.1588</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A28">
         <v>270</v>
       </c>
@@ -961,7 +975,7 @@
         <v>0.1067</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A29">
         <v>300</v>
       </c>
@@ -981,7 +995,7 @@
         <v>8.72E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A30">
         <v>330</v>
       </c>

</xml_diff>